<commit_message>
code updated 6/29; fixed heatmaps; started to create panel data
</commit_message>
<xml_diff>
--- a/GB_RPS Hard Code.xlsx
+++ b/GB_RPS Hard Code.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfc87df69086cb6c/Desktop/Green Bonds Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A1AC890-B7BF-40BF-AA96-865A19FC2583}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38D4A815-FF28-45F4-B207-4090A90134AE}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{D2DDFB62-C7BB-4467-AE1B-39ECA8DDC367}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2DDFB62-C7BB-4467-AE1B-39ECA8DDC367}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -60,9 +59,6 @@
     <t>Connecticut</t>
   </si>
   <si>
-    <t>Deleware</t>
-  </si>
-  <si>
     <t>Florida</t>
   </si>
   <si>
@@ -96,9 +92,6 @@
     <t>Maryland</t>
   </si>
   <si>
-    <t>Massachussetts</t>
-  </si>
-  <si>
     <t>Michigan</t>
   </si>
   <si>
@@ -202,6 +195,12 @@
   </si>
   <si>
     <t>Municipal Year</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>Delaware</t>
   </si>
 </sst>
 </file>
@@ -604,19 +603,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -627,13 +626,13 @@
         <v>2022</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -650,7 +649,7 @@
         <v>2006</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -664,10 +663,10 @@
         <v>2020</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -684,7 +683,7 @@
         <v>2002</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -701,7 +700,7 @@
         <v>2004</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -718,15 +717,15 @@
         <v>1998</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C8" s="3">
         <v>2019</v>
@@ -735,29 +734,29 @@
         <v>2005</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="3">
         <v>2019</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="3">
         <v>2016</v>
@@ -766,32 +765,32 @@
         <v>2018</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3">
         <v>2021</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="3">
         <v>2019</v>
@@ -803,12 +802,12 @@
         <v>2001</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="3">
         <v>2022</v>
@@ -820,12 +819,12 @@
         <v>2011</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3">
         <v>2017</v>
@@ -837,12 +836,12 @@
         <v>1983</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="3">
         <v>2016</v>
@@ -859,7 +858,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="3">
         <v>2018</v>
@@ -868,15 +867,15 @@
         <v>2022</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="3">
         <v>2021</v>
@@ -885,15 +884,15 @@
         <v>2022</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="3">
         <v>2017</v>
@@ -905,12 +904,12 @@
         <v>1999</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="3">
         <v>2021</v>
@@ -922,12 +921,12 @@
         <v>2004</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="B20" s="3">
         <v>2014</v>
@@ -939,12 +938,12 @@
         <v>1997</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21" s="3">
         <v>2018</v>
@@ -956,12 +955,12 @@
         <v>2008</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B22" s="3">
         <v>2021</v>
@@ -973,52 +972,52 @@
         <v>2007</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B23" s="3">
         <v>2021</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B24" s="3">
         <v>2021</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D24" s="3">
         <v>2007</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B25" s="3">
         <v>2023</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D25" s="3">
         <v>2005</v>
@@ -1029,27 +1028,27 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B26" s="3">
         <v>2022</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C27" s="3">
         <v>2017</v>
@@ -1058,29 +1057,29 @@
         <v>1997</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D28" s="3">
         <v>2007</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B29" s="3">
         <v>2019</v>
@@ -1092,12 +1091,12 @@
         <v>1991</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B30" s="3">
         <v>2019</v>
@@ -1109,12 +1108,12 @@
         <v>2002</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B31" s="3">
         <v>2014</v>
@@ -1126,12 +1125,12 @@
         <v>2004</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B32" s="3">
         <v>2018</v>
@@ -1143,18 +1142,18 @@
         <v>2007</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B33" s="3">
         <v>2022</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D33" s="3">
         <v>2007</v>
@@ -1165,7 +1164,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B34" s="3">
         <v>2019</v>
@@ -1177,18 +1176,18 @@
         <v>2008</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B35" s="3">
         <v>2021</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D35" s="3">
         <v>2010</v>
@@ -1199,7 +1198,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B36" s="3">
         <v>2021</v>
@@ -1211,29 +1210,29 @@
         <v>2007</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B37" s="3">
         <v>2019</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D37" s="3">
         <v>2004</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B38" s="3">
         <v>2018</v>
@@ -1245,12 +1244,12 @@
         <v>2004</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B39" s="3">
         <v>2022</v>
@@ -1262,18 +1261,18 @@
         <v>2014</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B40" s="3">
         <v>2018</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D40" s="3">
         <v>2008</v>
@@ -1284,7 +1283,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B41" s="3">
         <v>2023</v>
@@ -1293,15 +1292,15 @@
         <v>2017</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B42" s="3">
         <v>2020</v>
@@ -1313,15 +1312,15 @@
         <v>1999</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C43" s="3">
         <v>2014</v>
@@ -1330,15 +1329,15 @@
         <v>2008</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C44" s="3">
         <v>2015</v>
@@ -1347,12 +1346,12 @@
         <v>2005</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B45" s="3">
         <v>2018</v>
@@ -1364,15 +1363,15 @@
         <v>2020</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C46" s="3">
         <v>2015</v>
@@ -1381,15 +1380,15 @@
         <v>2006</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C47" s="3">
         <v>2021</v>
@@ -1403,7 +1402,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B48" s="3">
         <v>2021</v>
@@ -1420,19 +1419,19 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data cleaning finished, panel.csv created
</commit_message>
<xml_diff>
--- a/GB_RPS Hard Code.xlsx
+++ b/GB_RPS Hard Code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfc87df69086cb6c/Desktop/Green Bonds Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38D4A815-FF28-45F4-B207-4090A90134AE}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A2339B4-8D48-4D4C-90ED-C14223F51C47}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2DDFB62-C7BB-4467-AE1B-39ECA8DDC367}"/>
   </bookViews>
@@ -1116,10 +1116,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="3">
+        <v>2020</v>
+      </c>
+      <c r="C31" s="3">
         <v>2014</v>
-      </c>
-      <c r="C31" s="3">
-        <v>2020</v>
       </c>
       <c r="D31" s="3">
         <v>2004</v>

</xml_diff>

<commit_message>
fixed commenting on R-file
</commit_message>
<xml_diff>
--- a/GB_RPS Hard Code.xlsx
+++ b/GB_RPS Hard Code.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfc87df69086cb6c/Desktop/Green Bonds Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A2339B4-8D48-4D4C-90ED-C14223F51C47}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="8_{45399E63-9470-4378-9C44-D99E3C3F3DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE77EC0D-1A6A-406C-BF8B-4710562CF51E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2DDFB62-C7BB-4467-AE1B-39ECA8DDC367}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{D2DDFB62-C7BB-4467-AE1B-39ECA8DDC367}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
   <si>
     <t>Alabama</t>
   </si>
@@ -860,8 +860,8 @@
       <c r="A16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="3">
-        <v>2018</v>
+      <c r="B16" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="C16" s="3">
         <v>2022</v>
@@ -997,7 +997,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="3">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>49</v>
@@ -1030,8 +1030,8 @@
       <c r="A26" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="3">
-        <v>2022</v>
+      <c r="B26" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>49</v>
@@ -1150,7 +1150,7 @@
         <v>29</v>
       </c>
       <c r="B33" s="3">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>49</v>
@@ -1220,8 +1220,8 @@
       <c r="B37" s="3">
         <v>2019</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>49</v>
+      <c r="C37" s="3">
+        <v>2019</v>
       </c>
       <c r="D37" s="3">
         <v>2004</v>
@@ -1340,7 +1340,7 @@
         <v>49</v>
       </c>
       <c r="C44" s="3">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="D44" s="3">
         <v>2005</v>
@@ -1408,7 +1408,7 @@
         <v>2021</v>
       </c>
       <c r="C48" s="3">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D48" s="3">
         <v>1998</v>

</xml_diff>